<commit_message>
Windows build (hidden: analysis,mm,monitor)
</commit_message>
<xml_diff>
--- a/files/vol_marks.xlsx
+++ b/files/vol_marks.xlsx
@@ -55245,156 +55245,155 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultColWidth="8.82421875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>9</v>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>PAIRS</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>TENORS</t>
+        </is>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>14</v>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>USDJPY</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1w</t>
+        </is>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>18</v>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>USDCNH</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2w</t>
+        </is>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>19</v>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>USDCNY</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>3w</t>
+        </is>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>20</v>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>EURUSD</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>1m</t>
+        </is>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>21</v>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>GBPUSD</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2m</t>
+        </is>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>22</v>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>AUDUSD</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>3m</t>
+        </is>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>23</v>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>NZDUSD</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>6m</t>
+        </is>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I9" s="2" t="s">
-        <v>24</v>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>EURJPY</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>9m</t>
+        </is>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I10" s="2" t="s">
-        <v>25</v>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>AUDJPY</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>1y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>EURGBP</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>GBPNZD</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>EURCNH</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>GBPCNH</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Windows build (hidden: analysis,mm,monitor,listed)
</commit_message>
<xml_diff>
--- a/files/vol_marks.xlsx
+++ b/files/vol_marks.xlsx
@@ -30,6 +30,9 @@
     <sheet name="EVENTS" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="Vega Weights" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="BANDS" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="PEG_BANDS" sheetId="25" r:id="rIdCfg25"/>
+    <sheet name="KACE_SPREADS" sheetId="26" r:id="rIdCfg26"/>
+    <sheet name="HOLIDAYS" sheetId="27" r:id="rIdCfg27"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -7143,6 +7146,650 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="78" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Managed / pegged trading bands: pair, lower, upper, note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># These are policy settings, not market data. Check them against the central</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># bank before use, and delete a pair whose regime changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># A band here means a HARD, defended range for the spot. Only list a pair on</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># this tab if that is true: the model gives strikes outside the band zero</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># in-band value, which is right for a defended peg and wrong for anything else.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Not to be confused with the BANDS tab, which is the marking *treatment* for a</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># pegged pair -- hazard, jump sizes, blend. The defended range itself is here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pair</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">lower</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">upper</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">note</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USDHKD</t>
+        </is>
+      </c>
+      <c r="B13">
+        <v>7.75</v>
+      </c>
+      <c r="C13">
+        <v>7.85</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HKMA Convertibility Undertakings under the Linked Exchange Rate System</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Deliberately NOT listed:</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#   USDCNY - the +/-2% limit is around a daily fixing, so the band moves every</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#            day and is not a fixed range for a multi-month option.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#   USDCNH - offshore, not subject to the onshore limit at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#   DKK    - ERM II central rate 7.46038 with a +/-2.25% formal band, but the</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#            Nationalbank runs a far tighter de facto range; add it only with</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#            a range you are prepared to defend.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># The kACE feed: which tenors are posted as pillars, and the ATM bid/offer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># width at each, in volatility points.  Read by volkit/kace.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># The tenors listed for a pair are exactly the pillars posted for it, so a</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># pair with no rows here cannot be posted, and a tenor listed here with no</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># wing marks in the workbook is refused by name.  O/N is the one-day option</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># and borrows the shortest quoted tenor's wings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># A day between two pillars takes the spread of the earlier one; a day before</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># the O/N expiry takes O/N's.  These rows are the USDCNH sheet's column L.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pair</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tenor</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spread</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USDCNH</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O/N</t>
+        </is>
+      </c>
+      <c r="C12">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USDCNH</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1W</t>
+        </is>
+      </c>
+      <c r="C13">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USDCNH</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2W</t>
+        </is>
+      </c>
+      <c r="C14">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USDCNH</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1M</t>
+        </is>
+      </c>
+      <c r="C15">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USDCNH</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2M</t>
+        </is>
+      </c>
+      <c r="C16">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USDCNH</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3M</t>
+        </is>
+      </c>
+      <c r="C17">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USDCNH</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6M</t>
+        </is>
+      </c>
+      <c r="C18">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USDCNH</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9M</t>
+        </is>
+      </c>
+      <c r="C19">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USDCNH</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1Y</t>
+        </is>
+      </c>
+      <c r="C20">
+        <v>0.2</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Holiday dates no rule derives: country, date, remove.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Lunar-calendar holidays are published annually and cannot be worked out from</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># rules, so they are listed here. A row with remove = yes takes a date away</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># that the built-in rules would otherwise make a holiday.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Dates are YYYY-MM-DD. A '#' in the first column makes the whole row a note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">country</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">date</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">remove</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Chinese New Year 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CN</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-01-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CN</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-01-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CN</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-01-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CN</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-01-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CN</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-02-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CN</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-02-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># Chinese New Year 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CN</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CN</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CN</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CN</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CN</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-20</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
kACE spreads become tiers; Config workbook card folds; drop the premium label
</commit_message>
<xml_diff>
--- a/files/vol_marks.xlsx
+++ b/files/vol_marks.xlsx
@@ -7332,12 +7332,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="102" min="1" max="1"/>
-    <col width="10" customWidth="1" style="102" min="2" max="2"/>
-    <col width="10" customWidth="1" style="102" min="3" max="3"/>
+    <col width="10" customWidth="1" style="102" min="2" max="4"/>
+    <col width="30" customWidth="1" style="102" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7364,28 +7364,28 @@
     <row r="4">
       <c r="A4" s="99" t="inlineStr">
         <is>
-          <t># The tenors listed for a pair are exactly the pillars posted for it, so a</t>
+          <t># One row per tenor -- those are the pillars posted, so a tab with no rows</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="99" t="inlineStr">
         <is>
-          <t># pair with no rows here cannot be posted, and a tenor listed here with no</t>
+          <t># cannot be posted, and a tenor listed here with no wing marks in the</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="99" t="inlineStr">
         <is>
-          <t># wing marks in the workbook is refused by name.  O/N is the one-day option</t>
+          <t># workbook is refused by name.  O/N is the one-day option and borrows the</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="99" t="inlineStr">
         <is>
-          <t># and borrows the shortest quoted tenor's wings.</t>
+          <t># shortest quoted tenor's wings.</t>
         </is>
       </c>
     </row>
@@ -7399,171 +7399,238 @@
     <row r="9">
       <c r="A9" s="99" t="inlineStr">
         <is>
-          <t># A day between two pillars takes the spread of the earlier one; a day before</t>
+          <t># One column per spreading TIER: 'default', plus whatever else the desk</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="99" t="inlineStr">
         <is>
-          <t># the O/N expiry takes O/N's.  These rows are the USDCNH sheet's column L.</t>
+          <t># names.  A tier is a quoting policy and not a currency -- the pair is</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="99" t="inlineStr">
         <is>
-          <t>pair</t>
-        </is>
-      </c>
-      <c r="B11" s="99" t="inlineStr">
-        <is>
-          <t>tenor</t>
-        </is>
-      </c>
-      <c r="C11" s="99" t="inlineStr">
-        <is>
-          <t>spread</t>
+          <t># chosen on the kACE feed screen beside the tier -- and a cell a tier</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="99" t="inlineStr">
         <is>
-          <t>USDCNH</t>
-        </is>
-      </c>
-      <c r="B12" s="99" t="inlineStr">
-        <is>
-          <t>O/N</t>
-        </is>
-      </c>
-      <c r="C12" s="99" t="n">
-        <v>1</v>
+          <t># leaves blank takes 'default' for that tenor.  Tiers are added, edited</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="99" t="inlineStr">
         <is>
-          <t>USDCNH</t>
-        </is>
-      </c>
-      <c r="B13" s="99" t="inlineStr">
-        <is>
-          <t>1W</t>
-        </is>
-      </c>
-      <c r="C13" s="99" t="n">
-        <v>0.8</v>
+          <t># and removed in the Config window, and reach this file with the marks.</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="99" t="inlineStr">
         <is>
-          <t>USDCNH</t>
-        </is>
-      </c>
-      <c r="B14" s="99" t="inlineStr">
-        <is>
-          <t>2W</t>
-        </is>
-      </c>
-      <c r="C14" s="99" t="n">
-        <v>0.6</v>
+          <t>#</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="99" t="inlineStr">
         <is>
-          <t>USDCNH</t>
-        </is>
-      </c>
-      <c r="B15" s="99" t="inlineStr">
-        <is>
-          <t>1M</t>
-        </is>
-      </c>
-      <c r="C15" s="99" t="n">
-        <v>0.4</v>
+          <t># A day between two pillars takes the spread of the earlier one; a day before</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="99" t="inlineStr">
         <is>
-          <t>USDCNH</t>
-        </is>
-      </c>
-      <c r="B16" s="99" t="inlineStr">
-        <is>
-          <t>2M</t>
-        </is>
-      </c>
-      <c r="C16" s="99" t="n">
-        <v>0.3</v>
+          <t># the O/N expiry takes O/N's.  The 'default' column is the USDCNH sheet's</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="99" t="inlineStr">
         <is>
-          <t>USDCNH</t>
-        </is>
-      </c>
-      <c r="B17" s="99" t="inlineStr">
-        <is>
-          <t>3M</t>
-        </is>
-      </c>
-      <c r="C17" s="99" t="n">
-        <v>0.3</v>
+          <t># column L, which is where this table started.</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="99" t="inlineStr">
         <is>
-          <t>USDCNH</t>
+          <t>tenor</t>
         </is>
       </c>
       <c r="B18" s="99" t="inlineStr">
         <is>
-          <t>6M</t>
-        </is>
-      </c>
-      <c r="C18" s="99" t="n">
-        <v>0.2</v>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="C18" s="99" t="inlineStr">
+        <is>
+          <t>wide</t>
+        </is>
+      </c>
+      <c r="D18" s="99" t="inlineStr">
+        <is>
+          <t>thin</t>
+        </is>
+      </c>
+      <c r="E18" s="99" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="99" t="inlineStr">
         <is>
-          <t>USDCNH</t>
-        </is>
-      </c>
-      <c r="B19" s="99" t="inlineStr">
-        <is>
-          <t>9M</t>
-        </is>
+          <t>O/N</t>
+        </is>
+      </c>
+      <c r="B19" s="99" t="n">
+        <v>1</v>
       </c>
       <c r="C19" s="99" t="n">
-        <v>0.2</v>
+        <v>1.5</v>
+      </c>
+      <c r="D19" s="99" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="99" t="inlineStr">
         <is>
-          <t>USDCNH</t>
-        </is>
-      </c>
-      <c r="B20" s="99" t="inlineStr">
+          <t>1W</t>
+        </is>
+      </c>
+      <c r="B20" s="99" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C20" s="99" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D20" s="99" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="99" t="inlineStr">
+        <is>
+          <t>2W</t>
+        </is>
+      </c>
+      <c r="B21" s="99" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C21" s="99" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D21" s="99" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="99" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="B22" s="99" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C22" s="99" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D22" s="99" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="99" t="inlineStr">
+        <is>
+          <t>2M</t>
+        </is>
+      </c>
+      <c r="B23" s="99" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C23" s="99" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D23" s="99" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="99" t="inlineStr">
+        <is>
+          <t>3M</t>
+        </is>
+      </c>
+      <c r="B24" s="99" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C24" s="99" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D24" s="99" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="99" t="inlineStr">
+        <is>
+          <t>6M</t>
+        </is>
+      </c>
+      <c r="B25" s="99" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C25" s="99" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D25" s="99" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="99" t="inlineStr">
+        <is>
+          <t>9M</t>
+        </is>
+      </c>
+      <c r="B26" s="99" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C26" s="99" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D26" s="99" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="99" t="inlineStr">
         <is>
           <t>1Y</t>
         </is>
       </c>
-      <c r="C20" s="99" t="n">
+      <c r="B27" s="99" t="n">
         <v>0.2</v>
       </c>
+      <c r="C27" s="99" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D27" s="99" t="n">
+        <v>0.15</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>